<commit_message>
Updated Velocity and Burndown Chart
</commit_message>
<xml_diff>
--- a/Evidence/PMC/Burndown_Chart.xlsx
+++ b/Evidence/PMC/Burndown_Chart.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanil\Projects\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanil\Projects\CO3095 YEAR 3 SOFTWARE\Evidence\PMC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17408144-BE8C-4429-BD75-DFF6B96613A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A7D38AA-B9A1-4D33-BB6D-8FB27312E5AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D9FB4B47-6754-40F5-BCDE-6069D18C138F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Phase</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t>Achieved</t>
+  </si>
+  <si>
+    <t>Velocity</t>
   </si>
 </sst>
 </file>
@@ -338,7 +341,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-GB"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -626,6 +629,9 @@
                 <c:pt idx="0">
                   <c:v>203</c:v>
                 </c:pt>
+                <c:pt idx="1">
+                  <c:v>168</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -633,6 +639,144 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-609C-45E0-9D1A-DDF85EE35ADD}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet1!$A$14</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Velocity</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="t"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet1!$B$11:$F$11</c:f>
+              <c:strCache>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>Kick-off</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>End of Sprint 1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>End of Sprint 2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>End of Sprint 3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>End of Sprint 4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet1!$B$14:$F$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="1">
+                  <c:v>35</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-5054-44F0-B9AD-5ABD3803903B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -792,7 +936,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-GB"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1519,8 +1663,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{659A0515-EAB0-4206-BDC6-689C88D6D3F4}" name="Table2" displayName="Table2" ref="A11:F13" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
-  <autoFilter ref="A11:F13" xr:uid="{659A0515-EAB0-4206-BDC6-689C88D6D3F4}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{659A0515-EAB0-4206-BDC6-689C88D6D3F4}" name="Table2" displayName="Table2" ref="A11:F14" totalsRowShown="0" headerRowDxfId="7" dataDxfId="6">
+  <autoFilter ref="A11:F14" xr:uid="{659A0515-EAB0-4206-BDC6-689C88D6D3F4}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -1529,12 +1673,12 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{1CE1EED2-9721-4586-B2A3-E175F48EA0B4}" name="Phase" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{5CBACC87-8E87-4539-9CFB-C2CFF2D63E5A}" name="Kick-off" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{5E790456-8B00-452C-B5DD-67A19EFE80A7}" name="End of Sprint 1" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{EFE9C296-5F92-42C8-B101-6CC19BD07D4B}" name="End of Sprint 2" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{3B7F9E33-A3B0-4A52-9BAB-BE364ED2DD72}" name="End of Sprint 3" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{3DBA53A6-7422-42F3-9A4C-B23066F65F0E}" name="End of Sprint 4" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{1CE1EED2-9721-4586-B2A3-E175F48EA0B4}" name="Phase" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{5CBACC87-8E87-4539-9CFB-C2CFF2D63E5A}" name="Kick-off" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{5E790456-8B00-452C-B5DD-67A19EFE80A7}" name="End of Sprint 1" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{EFE9C296-5F92-42C8-B101-6CC19BD07D4B}" name="End of Sprint 2" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{3B7F9E33-A3B0-4A52-9BAB-BE364ED2DD72}" name="End of Sprint 3" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{3DBA53A6-7422-42F3-9A4C-B23066F65F0E}" name="End of Sprint 4" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -1857,7 +2001,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C08A02C7-E5CB-4902-90F9-E81E04608F5F}">
-  <dimension ref="A11:F15"/>
+  <dimension ref="A11:F14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" customWidth="1"/>
@@ -1869,72 +2013,67 @@
   </cols>
   <sheetData>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>0</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>1</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>2</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" t="s">
         <v>3</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" t="s">
         <v>4</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>6</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12">
         <v>203</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12">
         <v>168</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12">
         <v>128</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12">
         <v>70</v>
       </c>
-      <c r="F12" s="1">
+      <c r="F12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13">
         <v>203</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
+      <c r="C13">
+        <v>168</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1"/>
+      <c r="A14" s="1" t="s">
+        <v>8</v>
+      </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
+      <c r="C14" s="1">
+        <v>35</v>
+      </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated Burndown Chart For Sprint 2 Metrics
</commit_message>
<xml_diff>
--- a/Evidence/PMC/Burndown_Chart.xlsx
+++ b/Evidence/PMC/Burndown_Chart.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanil\Projects\CO3095 YEAR 3 SOFTWARE\Evidence\PMC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A7D38AA-B9A1-4D33-BB6D-8FB27312E5AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C406162-2CA8-4FC5-88BE-931280A47B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D9FB4B47-6754-40F5-BCDE-6069D18C138F}"/>
+    <workbookView xWindow="2124" yWindow="2124" windowWidth="17280" windowHeight="8880" xr2:uid="{D9FB4B47-6754-40F5-BCDE-6069D18C138F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -98,9 +98,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -632,6 +631,9 @@
                 <c:pt idx="1">
                   <c:v>168</c:v>
                 </c:pt>
+                <c:pt idx="2">
+                  <c:v>128</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -769,6 +771,9 @@
                 <c:ptCount val="5"/>
                 <c:pt idx="1">
                   <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>40</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2062,18 +2067,20 @@
       <c r="C13">
         <v>168</v>
       </c>
+      <c r="D13">
+        <v>128</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1">
+      <c r="C14">
         <v>35</v>
       </c>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
-      <c r="F14" s="1"/>
+      <c r="D14">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated Burndown Chart with sprint 3 metrics
</commit_message>
<xml_diff>
--- a/Evidence/PMC/Burndown_Chart.xlsx
+++ b/Evidence/PMC/Burndown_Chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanil\Projects\CO3095 YEAR 3 SOFTWARE\Evidence\PMC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C406162-2CA8-4FC5-88BE-931280A47B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CED20514-4065-402E-A7CA-EBE99279A68D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2124" yWindow="2124" windowWidth="17280" windowHeight="8880" xr2:uid="{D9FB4B47-6754-40F5-BCDE-6069D18C138F}"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{D9FB4B47-6754-40F5-BCDE-6069D18C138F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -634,6 +634,9 @@
                 <c:pt idx="2">
                   <c:v>128</c:v>
                 </c:pt>
+                <c:pt idx="3">
+                  <c:v>70</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -774,6 +777,9 @@
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>58</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2070,6 +2076,9 @@
       <c r="D13">
         <v>128</v>
       </c>
+      <c r="E13">
+        <v>70</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -2081,6 +2090,9 @@
       <c r="D14">
         <v>40</v>
       </c>
+      <c r="E14">
+        <v>58</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated Burndown Chart With Sprint 4 metrics.
</commit_message>
<xml_diff>
--- a/Evidence/PMC/Burndown_Chart.xlsx
+++ b/Evidence/PMC/Burndown_Chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanil\Projects\CO3095 YEAR 3 SOFTWARE\Evidence\PMC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CED20514-4065-402E-A7CA-EBE99279A68D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6780F68D-EEF1-4493-BD42-EA15EDA13D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{D9FB4B47-6754-40F5-BCDE-6069D18C138F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D9FB4B47-6754-40F5-BCDE-6069D18C138F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -637,6 +637,9 @@
                 <c:pt idx="3">
                   <c:v>70</c:v>
                 </c:pt>
+                <c:pt idx="4">
+                  <c:v>0</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -780,6 +783,9 @@
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>58</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>70</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2079,6 +2085,9 @@
       <c r="E13">
         <v>70</v>
       </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -2092,6 +2101,9 @@
       </c>
       <c r="E14">
         <v>58</v>
+      </c>
+      <c r="F14">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance player queue functionality with improved state validation and error handling
</commit_message>
<xml_diff>
--- a/Evidence/PMC/Burndown_Chart.xlsx
+++ b/Evidence/PMC/Burndown_Chart.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanil\Projects\CO3095 YEAR 3 SOFTWARE\Evidence\PMC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6780F68D-EEF1-4493-BD42-EA15EDA13D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{991393F3-961C-4F7D-9FFB-BA39E18DA019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D9FB4B47-6754-40F5-BCDE-6069D18C138F}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{D9FB4B47-6754-40F5-BCDE-6069D18C138F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Changes to Burndown Chart for better readability.
</commit_message>
<xml_diff>
--- a/Evidence/PMC/Burndown_Chart.xlsx
+++ b/Evidence/PMC/Burndown_Chart.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanil\Projects\CO3095 YEAR 3 SOFTWARE\Evidence\PMC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neelp\PycharmProjects\CO3095-Group-16-Music-Player-Application\Evidence\PMC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{991393F3-961C-4F7D-9FFB-BA39E18DA019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D23610A8-47AD-480C-92F6-CF06887490E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="360" windowWidth="23256" windowHeight="12456" xr2:uid="{D9FB4B47-6754-40F5-BCDE-6069D18C138F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D9FB4B47-6754-40F5-BCDE-6069D18C138F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -389,6 +389,116 @@
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-4.9691021446746669E-2"/>
+                  <c:y val="7.0132790048269222E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000009-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-6.2413667757179207E-2"/>
+                  <c:y val="7.0132790048269222E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-7.1501272264631044E-2"/>
+                  <c:y val="7.4138665753200841E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-8.7350054525627177E-2"/>
+                  <c:y val="6.0387787693634409E-3"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-3.9585605234460329E-2"/>
+                  <c:y val="-5.8055232509542344E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000D-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -479,13 +589,13 @@
                   <c:v>203</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>168</c:v>
+                  <c:v>165</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>128</c:v>
+                  <c:v>125</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>70</c:v>
+                  <c:v>68</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -539,6 +649,116 @@
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:dLbl>
+              <c:idx val="0"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="8.4696474009450778E-3"/>
+                  <c:y val="-6.2061108214473956E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000008-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-9.7055616139585608E-3"/>
+                  <c:y val="-6.6066983919405561E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="2.3009814612868114E-2"/>
+                  <c:y val="-0.10211986526379006"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000002-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-1.9265721555799225E-3"/>
+                  <c:y val="-0.11013161667365337"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000004-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="1.1304980007270083E-2"/>
+                  <c:y val="-6.6066983919405714E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000C-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -689,6 +909,94 @@
             </c:spPr>
           </c:marker>
           <c:dLbls>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-2.3736822973464196E-2"/>
+                  <c:y val="-5.8055232509542413E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000B-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-2.7371864776444994E-2"/>
+                  <c:y val="-6.2061108214474026E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{0000000A-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="3"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-2.191930207197396E-2"/>
+                  <c:y val="6.2121038638406005E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000006-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="4"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-1.4649218466012359E-2"/>
+                  <c:y val="-7.4078735329268869E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="r"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000007-E3F8-4680-B397-92E2C50AB583}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -2019,17 +2327,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C08A02C7-E5CB-4902-90F9-E81E04608F5F}">
   <dimension ref="A11:F14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" customWidth="1"/>
-    <col min="2" max="2" width="9.33203125" customWidth="1"/>
+    <col min="1" max="1" width="8.90625" customWidth="1"/>
+    <col min="2" max="2" width="9.36328125" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="5" width="15.88671875" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" customWidth="1"/>
-    <col min="7" max="7" width="17.21875" customWidth="1"/>
+    <col min="4" max="5" width="15.90625" customWidth="1"/>
+    <col min="6" max="6" width="14.6328125" customWidth="1"/>
+    <col min="7" max="7" width="17.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -2049,7 +2357,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>6</v>
       </c>
@@ -2057,19 +2365,19 @@
         <v>203</v>
       </c>
       <c r="C12">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D12">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="E12">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F12">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -2089,7 +2397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Updated Burndown Chart with correct figures
</commit_message>
<xml_diff>
--- a/Evidence/PMC/Burndown_Chart.xlsx
+++ b/Evidence/PMC/Burndown_Chart.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\neelp\PycharmProjects\CO3095-Group-16-Music-Player-Application\Evidence\PMC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D23610A8-47AD-480C-92F6-CF06887490E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{007221D6-842B-46EA-9A62-EE4A4F04DAB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{D9FB4B47-6754-40F5-BCDE-6069D18C138F}"/>
   </bookViews>
@@ -393,8 +393,8 @@
               <c:idx val="0"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-4.9691021446746669E-2"/>
-                  <c:y val="7.0132790048269222E-2"/>
+                  <c:x val="1.2320261602169678E-2"/>
+                  <c:y val="-4.452128885815114E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -415,8 +415,8 @@
               <c:idx val="1"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-6.2413667757179207E-2"/>
-                  <c:y val="7.0132790048269222E-2"/>
+                  <c:x val="-4.0239859433353274E-4"/>
+                  <c:y val="-7.7279578785138178E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -437,8 +437,8 @@
               <c:idx val="2"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-7.1501272264631044E-2"/>
-                  <c:y val="7.4138665753200841E-2"/>
+                  <c:x val="-4.0183851063692287E-3"/>
+                  <c:y val="-7.3273781599578314E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -459,8 +459,8 @@
               <c:idx val="3"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-8.7350054525627177E-2"/>
-                  <c:y val="6.0387787693634409E-3"/>
+                  <c:x val="-7.1001379385616905E-3"/>
+                  <c:y val="-8.8141402319196649E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -589,13 +589,13 @@
                   <c:v>203</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>165</c:v>
+                  <c:v>170</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>125</c:v>
+                  <c:v>131</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>68</c:v>
+                  <c:v>72</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -653,8 +653,8 @@
               <c:idx val="0"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="8.4696474009450778E-3"/>
-                  <c:y val="-6.2061108214473956E-2"/>
+                  <c:x val="-4.4422392146190461E-2"/>
+                  <c:y val="0.16315208261795483"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -675,8 +675,8 @@
               <c:idx val="1"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-9.7055616139585608E-3"/>
-                  <c:y val="-6.6066983919405561E-2"/>
+                  <c:x val="-7.536457499341187E-2"/>
+                  <c:y val="0.11410363678278772"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -697,8 +697,8 @@
               <c:idx val="2"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="2.3009814612868114E-2"/>
-                  <c:y val="-0.10211986526379006"/>
+                  <c:x val="-7.5478745900797756E-2"/>
+                  <c:y val="7.39560310236482E-2"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -719,8 +719,8 @@
               <c:idx val="3"/>
               <c:layout>
                 <c:manualLayout>
-                  <c:x val="-1.9265721555799225E-3"/>
-                  <c:y val="-0.11013161667365337"/>
+                  <c:x val="-8.217648524502584E-2"/>
+                  <c:y val="4.5223206153141033E-3"/>
                 </c:manualLayout>
               </c:layout>
               <c:dLblPos val="r"/>
@@ -2365,13 +2365,13 @@
         <v>203</v>
       </c>
       <c r="C12">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D12">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="E12">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F12">
         <v>0</v>

</xml_diff>